<commit_message>
Substitui o motor de classificação pelo layout fixo "Cadastro de Produtos" dos clientes
Lê e devolve .xls/.xlsx com título mesclado, cabeçalho e aba intactos,
preenchendo automaticamente CFOP/CST/PIS-COFINS/IBS-CBS conforme a coluna
Tributação (Padrão A/B em lib/tables.ts) e sobrescritas por NCM (tabela
aberta NCM_OVERRIDES). Linhas já classificadas pelo cliente são apenas
validadas, nunca sobrescritas. Cada linha recebe Status e Observação.

Processamento em lotes com barra de progresso (testado com 60 mil linhas
sintéticas, ~5s ponta a ponta sem travar a UI). Tabela de resultado com
filtro por Status e paginação.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VvhY6TpV7FUhABWKSX2dNR
</commit_message>
<xml_diff>
--- a/public/planilha-modelo.xlsx
+++ b/public/planilha-modelo.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Produtos" sheetId="1" r:id="rId1"/>
+    <sheet name="Cadastro_de_Produtos" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,409 +397,1923 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:S32"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="24.83203125" customWidth="1"/>
-    <col min="11" max="11" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Código</v>
+        <v>Cadastro de Produtos</v>
       </c>
       <c r="B1" t="str">
-        <v>Descrição</v>
+        <v/>
       </c>
       <c r="C1" t="str">
-        <v>NCM</v>
+        <v/>
       </c>
       <c r="D1" t="str">
-        <v>Origem</v>
+        <v/>
       </c>
       <c r="E1" t="str">
-        <v>Tipo Operação</v>
+        <v/>
       </c>
       <c r="F1" t="str">
-        <v>Destino</v>
+        <v/>
       </c>
       <c r="G1" t="str">
-        <v>Destinatário</v>
+        <v/>
       </c>
       <c r="H1" t="str">
-        <v>ST Bahia</v>
+        <v/>
       </c>
       <c r="I1" t="str">
-        <v>Monofásico PIS/COFINS</v>
+        <v/>
       </c>
       <c r="J1" t="str">
-        <v>Isento PIS/COFINS</v>
+        <v/>
       </c>
       <c r="K1" t="str">
-        <v>Anexo LC 214/2025</v>
+        <v/>
+      </c>
+      <c r="L1" t="str">
+        <v/>
+      </c>
+      <c r="M1" t="str">
+        <v/>
+      </c>
+      <c r="N1" t="str">
+        <v/>
+      </c>
+      <c r="O1" t="str">
+        <v/>
+      </c>
+      <c r="P1" t="str">
+        <v/>
+      </c>
+      <c r="Q1" t="str">
+        <v/>
+      </c>
+      <c r="R1" t="str">
+        <v/>
+      </c>
+      <c r="S1" t="str">
+        <v/>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1001</v>
+        <v>Código</v>
       </c>
       <c r="B2" t="str">
-        <v>Parafuso sextavado zincado</v>
+        <v>Nome</v>
       </c>
       <c r="C2" t="str">
-        <v>73181500</v>
+        <v>Código de barras</v>
       </c>
       <c r="D2" t="str">
-        <v>0</v>
+        <v>UN</v>
       </c>
       <c r="E2" t="str">
-        <v>venda</v>
+        <v>Tributação</v>
       </c>
       <c r="F2" t="str">
-        <v>interna</v>
+        <v>Preço unit.</v>
       </c>
       <c r="G2" t="str">
-        <v>contribuinte</v>
+        <v>NCM</v>
       </c>
       <c r="H2" t="str">
-        <v>nao</v>
+        <v>CFOP SAIDAS</v>
       </c>
       <c r="I2" t="str">
-        <v>nao</v>
+        <v>ALIQ. FCP</v>
       </c>
       <c r="J2" t="str">
-        <v>nao</v>
+        <v>CST ICMS</v>
       </c>
       <c r="K2" t="str">
-        <v>nao</v>
+        <v>CST PIS/COFINS</v>
+      </c>
+      <c r="L2" t="str">
+        <v>PIS</v>
+      </c>
+      <c r="M2" t="str">
+        <v>COFINS</v>
+      </c>
+      <c r="N2" t="str">
+        <v>NAT. RECIETA</v>
+      </c>
+      <c r="O2" t="str">
+        <v>CST IBS/CBS</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Cclasstrib</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>RED. B.C.</v>
+      </c>
+      <c r="R2" t="str">
+        <v>IBS</v>
+      </c>
+      <c r="S2" t="str">
+        <v>CBS</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B3" t="str">
-        <v>Refrigerante de cola 2L</v>
+        <v>Parafuso sextavado zincado</v>
       </c>
       <c r="C3" t="str">
-        <v>22021000</v>
+        <v>7891000000011</v>
       </c>
       <c r="D3" t="str">
-        <v>0</v>
+        <v>UN</v>
       </c>
       <c r="E3" t="str">
-        <v>venda</v>
-      </c>
-      <c r="F3" t="str">
-        <v>interestadual</v>
+        <v>Tributado</v>
+      </c>
+      <c r="F3">
+        <v>3.5</v>
       </c>
       <c r="G3" t="str">
-        <v>consumidor_final</v>
+        <v>73181500</v>
       </c>
       <c r="H3" t="str">
-        <v>verificar</v>
+        <v/>
       </c>
       <c r="I3" t="str">
-        <v>sim</v>
+        <v/>
       </c>
       <c r="J3" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="K3" t="str">
-        <v>verificar</v>
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B4" t="str">
-        <v>Compra de material de escritório</v>
+        <v>Prego 18x30</v>
       </c>
       <c r="C4" t="str">
-        <v>48201000</v>
+        <v>7891000000028</v>
       </c>
       <c r="D4" t="str">
-        <v>0</v>
+        <v>CX</v>
       </c>
       <c r="E4" t="str">
-        <v>compra</v>
-      </c>
-      <c r="F4" t="str">
-        <v>interna</v>
+        <v>Tributado</v>
+      </c>
+      <c r="F4">
+        <v>12.9</v>
       </c>
       <c r="G4" t="str">
-        <v>contribuinte</v>
+        <v>73170010</v>
       </c>
       <c r="H4" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="I4" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="J4" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="K4" t="str">
-        <v>nao</v>
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="B5" t="str">
-        <v>Devolução de compra ao fornecedor</v>
+        <v>Pilha alcalina AA</v>
       </c>
       <c r="C5" t="str">
-        <v>73181500</v>
+        <v>7891000000035</v>
       </c>
       <c r="D5" t="str">
-        <v>0</v>
+        <v>PC</v>
       </c>
       <c r="E5" t="str">
-        <v>devolucao_compra</v>
-      </c>
-      <c r="F5" t="str">
-        <v>interestadual</v>
+        <v>Substituição tributária</v>
+      </c>
+      <c r="F5">
+        <v>4.2</v>
       </c>
       <c r="G5" t="str">
-        <v>contribuinte</v>
+        <v>85061000</v>
       </c>
       <c r="H5" t="str">
-        <v>verificar</v>
+        <v/>
       </c>
       <c r="I5" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="J5" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="K5" t="str">
-        <v>nao</v>
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="B6" t="str">
-        <v>Devolução de venda do cliente</v>
+        <v>Bateria 9V</v>
       </c>
       <c r="C6" t="str">
-        <v>73181500</v>
+        <v>7891000000042</v>
       </c>
       <c r="D6" t="str">
-        <v>0</v>
+        <v>PC</v>
       </c>
       <c r="E6" t="str">
-        <v>devolucao_venda</v>
-      </c>
-      <c r="F6" t="str">
-        <v>interna</v>
+        <v>Substituição tributária</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
       </c>
       <c r="G6" t="str">
-        <v>consumidor_final</v>
+        <v>85068000</v>
       </c>
       <c r="H6" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="I6" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="J6" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="K6" t="str">
-        <v>nao</v>
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B7" t="str">
-        <v>Transferência entre filiais</v>
+        <v>Carne bovina resfriada kg</v>
       </c>
       <c r="C7" t="str">
-        <v>73181500</v>
+        <v>7891000000059</v>
       </c>
       <c r="D7" t="str">
-        <v>0</v>
+        <v>KG</v>
       </c>
       <c r="E7" t="str">
-        <v>transferencia</v>
-      </c>
-      <c r="F7" t="str">
-        <v>interestadual</v>
+        <v>Tributado</v>
+      </c>
+      <c r="F7">
+        <v>32</v>
       </c>
       <c r="G7" t="str">
-        <v>contribuinte</v>
+        <v>02013000</v>
       </c>
       <c r="H7" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="I7" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="J7" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="K7" t="str">
-        <v>nao</v>
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B8" t="str">
-        <v>Bonificação a cliente</v>
+        <v>Carne suína resfriada kg</v>
       </c>
       <c r="C8" t="str">
-        <v>73181500</v>
+        <v>7891000000066</v>
       </c>
       <c r="D8" t="str">
-        <v>0</v>
+        <v>KG</v>
       </c>
       <c r="E8" t="str">
-        <v>bonificacao_doacao</v>
-      </c>
-      <c r="F8" t="str">
-        <v>interna</v>
+        <v>Tributado</v>
+      </c>
+      <c r="F8">
+        <v>18.5</v>
       </c>
       <c r="G8" t="str">
-        <v>contribuinte</v>
+        <v>02032900</v>
       </c>
       <c r="H8" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="I8" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="J8" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="K8" t="str">
-        <v>nao</v>
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B9" t="str">
-        <v>Remessa de equipamento para conserto</v>
+        <v>Frango inteiro congelado kg</v>
       </c>
       <c r="C9" t="str">
-        <v>84713012</v>
+        <v>7891000000073</v>
       </c>
       <c r="D9" t="str">
-        <v>0</v>
+        <v>KG</v>
       </c>
       <c r="E9" t="str">
-        <v>remessa_conserto</v>
-      </c>
-      <c r="F9" t="str">
-        <v>interestadual</v>
+        <v>Tributado</v>
+      </c>
+      <c r="F9">
+        <v>9.9</v>
       </c>
       <c r="G9" t="str">
-        <v>contribuinte</v>
+        <v>02071200</v>
       </c>
       <c r="H9" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="I9" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="J9" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="K9" t="str">
-        <v>nao</v>
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>1009</v>
+        <v>1027</v>
       </c>
       <c r="B10" t="str">
-        <v>Retorno de equipamento consertado</v>
+        <v>Carne caprina resfriada kg</v>
       </c>
       <c r="C10" t="str">
-        <v>84713012</v>
+        <v>7891000000264</v>
       </c>
       <c r="D10" t="str">
-        <v>0</v>
+        <v>KG</v>
       </c>
       <c r="E10" t="str">
-        <v>retorno_conserto</v>
-      </c>
-      <c r="F10" t="str">
-        <v>interestadual</v>
+        <v>Tributado</v>
+      </c>
+      <c r="F10">
+        <v>28</v>
       </c>
       <c r="G10" t="str">
-        <v>contribuinte</v>
+        <v>02042100</v>
       </c>
       <c r="H10" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="I10" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="J10" t="str">
-        <v>nao</v>
+        <v/>
       </c>
       <c r="K10" t="str">
-        <v>nao</v>
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>1008</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Xampu 350ml</v>
+      </c>
+      <c r="C11" t="str">
+        <v>7891000000080</v>
+      </c>
+      <c r="D11" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F11">
+        <v>14.9</v>
+      </c>
+      <c r="G11" t="str">
+        <v>33051000</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>1009</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Desodorante aerosol</v>
+      </c>
+      <c r="C12" t="str">
+        <v>7891000000097</v>
+      </c>
+      <c r="D12" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F12">
+        <v>11.5</v>
+      </c>
+      <c r="G12" t="str">
+        <v>33072010</v>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>1028</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Creme de pentear 500ml</v>
+      </c>
+      <c r="C13" t="str">
+        <v>7891000000271</v>
+      </c>
+      <c r="D13" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F13">
+        <v>13.2</v>
+      </c>
+      <c r="G13" t="str">
+        <v>33072090</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
         <v>1010</v>
       </c>
-      <c r="B11" t="str">
-        <v>Venda para órgão público</v>
-      </c>
-      <c r="C11" t="str">
-        <v>73181500</v>
-      </c>
-      <c r="D11" t="str">
-        <v>0</v>
-      </c>
-      <c r="E11" t="str">
-        <v>venda</v>
-      </c>
-      <c r="F11" t="str">
-        <v>interna</v>
-      </c>
-      <c r="G11" t="str">
-        <v>orgao_publico</v>
-      </c>
-      <c r="H11" t="str">
-        <v>nao</v>
-      </c>
-      <c r="I11" t="str">
-        <v>nao</v>
-      </c>
-      <c r="J11" t="str">
-        <v>nao</v>
-      </c>
-      <c r="K11" t="str">
-        <v>verificar</v>
+      <c r="B14" t="str">
+        <v>Escova dental macia</v>
+      </c>
+      <c r="C14" t="str">
+        <v>7891000000103</v>
+      </c>
+      <c r="D14" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F14">
+        <v>3.9</v>
+      </c>
+      <c r="G14" t="str">
+        <v>96032100</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>1011</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Inseticida aerosol 300ml</v>
+      </c>
+      <c r="C15" t="str">
+        <v>7891000000110</v>
+      </c>
+      <c r="D15" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F15">
+        <v>16.9</v>
+      </c>
+      <c r="G15" t="str">
+        <v>38089410</v>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>1012</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Produto tributado já classificado</v>
+      </c>
+      <c r="C16" t="str">
+        <v>7891000000127</v>
+      </c>
+      <c r="D16" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F16">
+        <v>20</v>
+      </c>
+      <c r="G16" t="str">
+        <v>39269090</v>
+      </c>
+      <c r="H16" t="str">
+        <v>5102</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v>000</v>
+      </c>
+      <c r="K16" t="str">
+        <v>01</v>
+      </c>
+      <c r="L16">
+        <v>1.65</v>
+      </c>
+      <c r="M16">
+        <v>7.6</v>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v>000</v>
+      </c>
+      <c r="P16" t="str">
+        <v>000001</v>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16">
+        <v>0.1</v>
+      </c>
+      <c r="S16">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>1013</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Produto com ST já classificado</v>
+      </c>
+      <c r="C17" t="str">
+        <v>7891000000134</v>
+      </c>
+      <c r="D17" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Substituição tributária</v>
+      </c>
+      <c r="F17">
+        <v>22</v>
+      </c>
+      <c r="G17" t="str">
+        <v>40169300</v>
+      </c>
+      <c r="H17" t="str">
+        <v>5405</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v>060</v>
+      </c>
+      <c r="K17" t="str">
+        <v>01</v>
+      </c>
+      <c r="L17">
+        <v>1.65</v>
+      </c>
+      <c r="M17">
+        <v>7.6</v>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v>000</v>
+      </c>
+      <c r="P17" t="str">
+        <v>000001</v>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17">
+        <v>0.1</v>
+      </c>
+      <c r="S17">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>1014</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Produto com cClassTrib de 7 dígitos (a mais)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>7891000000141</v>
+      </c>
+      <c r="D18" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F18">
+        <v>25</v>
+      </c>
+      <c r="G18" t="str">
+        <v>39269090</v>
+      </c>
+      <c r="H18" t="str">
+        <v>5102</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v>000</v>
+      </c>
+      <c r="K18" t="str">
+        <v>01</v>
+      </c>
+      <c r="L18">
+        <v>1.65</v>
+      </c>
+      <c r="M18">
+        <v>7.6</v>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v>000</v>
+      </c>
+      <c r="P18" t="str">
+        <v>2000003</v>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18">
+        <v>0.1</v>
+      </c>
+      <c r="S18">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>1015</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Produto com cClassTrib de 5 dígitos (a menos)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>7891000000158</v>
+      </c>
+      <c r="D19" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F19">
+        <v>19</v>
+      </c>
+      <c r="G19" t="str">
+        <v>39269090</v>
+      </c>
+      <c r="H19" t="str">
+        <v>5102</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v>000</v>
+      </c>
+      <c r="K19" t="str">
+        <v>01</v>
+      </c>
+      <c r="L19">
+        <v>1.65</v>
+      </c>
+      <c r="M19">
+        <v>7.6</v>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v>000</v>
+      </c>
+      <c r="P19" t="str">
+        <v>20003</v>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19">
+        <v>0.1</v>
+      </c>
+      <c r="S19">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>1016</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Produto com cClassTrib de 7 dígitos (zero a mais)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>7891000000165</v>
+      </c>
+      <c r="D20" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F20">
+        <v>21</v>
+      </c>
+      <c r="G20" t="str">
+        <v>39269090</v>
+      </c>
+      <c r="H20" t="str">
+        <v>5102</v>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v>000</v>
+      </c>
+      <c r="K20" t="str">
+        <v>01</v>
+      </c>
+      <c r="L20">
+        <v>1.65</v>
+      </c>
+      <c r="M20">
+        <v>7.6</v>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v>000</v>
+      </c>
+      <c r="P20" t="str">
+        <v>0000001</v>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20">
+        <v>0.1</v>
+      </c>
+      <c r="S20">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>1017</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Produto com CST ICMS divergente</v>
+      </c>
+      <c r="C21" t="str">
+        <v>7891000000172</v>
+      </c>
+      <c r="D21" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F21">
+        <v>17</v>
+      </c>
+      <c r="G21" t="str">
+        <v>39269090</v>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v>40</v>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
+      <c r="S21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>1018</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Produto não tributado</v>
+      </c>
+      <c r="C22" t="str">
+        <v>7891000000189</v>
+      </c>
+      <c r="D22" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Não tributado</v>
+      </c>
+      <c r="F22">
+        <v>5</v>
+      </c>
+      <c r="G22" t="str">
+        <v>49019900</v>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>1019</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Produto isento</v>
+      </c>
+      <c r="C23" t="str">
+        <v>7891000000196</v>
+      </c>
+      <c r="D23" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Isento</v>
+      </c>
+      <c r="F23">
+        <v>6</v>
+      </c>
+      <c r="G23" t="str">
+        <v>49019900</v>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>1020</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Produto com tributação suspensa</v>
+      </c>
+      <c r="C24" t="str">
+        <v>7891000000202</v>
+      </c>
+      <c r="D24" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Suspenso</v>
+      </c>
+      <c r="F24">
+        <v>8</v>
+      </c>
+      <c r="G24" t="str">
+        <v>39269090</v>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>1021</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Envelope de papel</v>
+      </c>
+      <c r="C25" t="str">
+        <v>7891000000219</v>
+      </c>
+      <c r="D25" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F25">
+        <v>2.5</v>
+      </c>
+      <c r="G25" t="str">
+        <v>4820.20.00</v>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v/>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
+      <c r="S25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>1022</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Produto com NCM incompleto</v>
+      </c>
+      <c r="C26" t="str">
+        <v>7891000000226</v>
+      </c>
+      <c r="D26" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F26">
+        <v>10</v>
+      </c>
+      <c r="G26" t="str">
+        <v>16185</v>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v/>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>1023</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Produto sem NCM informado</v>
+      </c>
+      <c r="C27" t="str">
+        <v>7891000000233</v>
+      </c>
+      <c r="D27" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F27">
+        <v>12</v>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>1024</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Produto com PIS divergente</v>
+      </c>
+      <c r="C28" t="str">
+        <v>7891000000240</v>
+      </c>
+      <c r="D28" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F28">
+        <v>30</v>
+      </c>
+      <c r="G28" t="str">
+        <v>39269090</v>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28">
+        <v>2.5</v>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
+      <c r="S28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>1025</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Cadeira de escritório</v>
+      </c>
+      <c r="C29" t="str">
+        <v>7891000000257</v>
+      </c>
+      <c r="D29" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F29">
+        <v>350</v>
+      </c>
+      <c r="G29" t="str">
+        <v>94013000</v>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+      <c r="O29" t="str">
+        <v/>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
+      <c r="R29" t="str">
+        <v/>
+      </c>
+      <c r="S29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>1026</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Extensão elétrica 5m</v>
+      </c>
+      <c r="C30" t="str">
+        <v>7891000000301</v>
+      </c>
+      <c r="D30" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Substituição tributária</v>
+      </c>
+      <c r="F30">
+        <v>28</v>
+      </c>
+      <c r="G30" t="str">
+        <v>85446000</v>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v/>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
+        <v/>
+      </c>
+      <c r="O30" t="str">
+        <v/>
+      </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
+      <c r="R30" t="str">
+        <v/>
+      </c>
+      <c r="S30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>1029</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Produto com preenchimento parcial</v>
+      </c>
+      <c r="C31" t="str">
+        <v>7891000000288</v>
+      </c>
+      <c r="D31" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F31">
+        <v>15.5</v>
+      </c>
+      <c r="G31" t="str">
+        <v>39269090</v>
+      </c>
+      <c r="H31" t="str">
+        <v>5102</v>
+      </c>
+      <c r="I31" t="str">
+        <v/>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
+        <v/>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
+      <c r="N31" t="str">
+        <v/>
+      </c>
+      <c r="O31" t="str">
+        <v/>
+      </c>
+      <c r="P31" t="str">
+        <v/>
+      </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
+      <c r="R31" t="str">
+        <v/>
+      </c>
+      <c r="S31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>1030</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Produto com NAT. RECEITA divergente</v>
+      </c>
+      <c r="C32" t="str">
+        <v>7891000000295</v>
+      </c>
+      <c r="D32" t="str">
+        <v>UN</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Tributado</v>
+      </c>
+      <c r="F32">
+        <v>9.5</v>
+      </c>
+      <c r="G32" t="str">
+        <v>39269090</v>
+      </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
+        <v/>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
+      <c r="N32" t="str">
+        <v>999</v>
+      </c>
+      <c r="O32" t="str">
+        <v/>
+      </c>
+      <c r="P32" t="str">
+        <v/>
+      </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
+      <c r="R32" t="str">
+        <v/>
+      </c>
+      <c r="S32" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:S1"/>
+  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>